<commit_message>
fix(tex_reader): improve LaTeX parsing robustness and add auto column width
- Fix negative multirow handling: relocate content from bottom to top of merged range
- Fix \dagger/\dag replacement order to prevent "†ger" artifacts
- Fix superscript \text{} handling (MME^\text{P} → MMEP)
- Fix subscript regex to avoid matching multi-char like _stage
- Add escaped \& support in ampersand splitting
- Add \midrule[0.5pt] optional argument support
- Improve multicolumn/multirow regex for nested braces and optional args
- Convert logo commands to text labels ([Lang], [Img], [Vid])
- Add extensive LaTeX command cleanup (colors, rules, custom commands)
- writer: auto-adjust column widths, wrap text, rotation support
- writer: cap rowspan to avoid overlapping merges
- renderer: skip horizontal placeholder cells, auto-cmidrule
- utils: add em-dash to unicode-latex mapping
- Update table4 test fixture for makecell newline behavior

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/table4.xlsx
+++ b/tests/fixtures/table4.xlsx
@@ -50,10 +50,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -472,510 +475,514 @@
           <t>SEED-DV</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>Things-EEG</t>
-        </is>
-      </c>
-      <c r="M2" s="1" t="inlineStr">
-        <is>
-          <t>Faces-Houses</t>
-        </is>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
-        <is>
-          <t>Open-MIIR-P</t>
-        </is>
-      </c>
-      <c r="Q2" s="1" t="inlineStr">
-        <is>
-          <t>Open-MIIR-I</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Things-
+EEG</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Faces-
+Houses</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Open-
+MIIR-P</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Open-
+MIIR-I</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ConvFormer</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>.394±.005</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>.086±.001</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>.080±.004</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>.024±.000</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>.151±.003</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>.820±.013</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>.975±.005</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>.976±.002</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>CAFormer</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>.221±.003</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>.081±.003</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>.076±.002</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>.025±.001</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>.160±.009</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>.800±.012</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>.976±.006</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>.977±.002</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>ModernTCN</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>.339±.005</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>.079±.003</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>.074±.002</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>.040±.001</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>.123±.003</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>.835±.006</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>.964±.010</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>.935±.002</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>MedFormer</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>.212±.006</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>.089±.003</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>.085±.001</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>.025±.000</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>.045±.002</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>.756±.011</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>.948±.001</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>.941±.001</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>DeepConvNet</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>.053±.002</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>.053±.004</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>.052±.001</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>.029±.001</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>.091±.001</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>.822±.005</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>.896±.009</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>.789±.005</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>EEGNet</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>.060±.003</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>.071±.002</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>.082±.002</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>.046±.002</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>.070±.000</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>.830±.006</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>.915±.010</t>
         </is>
       </c>
-      <c r="Q9" s="3" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>.852±.006</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Conformer</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>.205±.003</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>.095±.002</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>.087±.002</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>.033±.002</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>.077±.002</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>.762±.001</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>.962±.013</t>
         </is>
       </c>
-      <c r="Q10" s="3" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>.930±.002</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>SPaRCNet</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>.026±.001</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>.005±.000</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>.005±.000</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>.026±.001</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>.189±.001</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>.805±.007</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>.969±.007</t>
         </is>
       </c>
-      <c r="Q11" s="3" t="inlineStr">
+      <c r="Q11" s="4" t="inlineStr">
         <is>
           <t>.948±.005</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>seegnificant</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>.053±.002</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>.831±.006</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>CBraMod</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>.084±.002</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>.077±.001</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>.026±.002</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>.975±.011</t>
         </is>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>.933±.008</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>NeuroSketch-Base</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>.472±.006</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>.111±.001</t>
         </is>
@@ -985,7 +992,7 @@
           <t>.103±.002</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>.045±.002</t>
         </is>
@@ -995,24 +1002,24 @@
           <t>.196±.002</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>.879±.008</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>.981±.010</t>
         </is>
       </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>.970±.002</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>NeuroSketch-Large</t>
         </is>
@@ -1027,7 +1034,7 @@
           <t>.116±.001</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>.095±.005</t>
         </is>
@@ -1037,7 +1044,7 @@
           <t>.047±.003</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>.177±.001</t>
         </is>

</xml_diff>